<commit_message>
feat: enhance unit upload process by supporting bulk uploads and improving error handling
</commit_message>
<xml_diff>
--- a/public/unit_upload_template.xlsx
+++ b/public/unit_upload_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\work\lenaAI\lenaai-website\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AD1EA71-7A35-4B4B-8395-376E14F01C16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B700EFB-E625-4D82-91A1-E36924E136C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2832" yWindow="2832" windowWidth="22656" windowHeight="12120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -97,9 +97,6 @@
     <t>Lake View Apartment</t>
   </si>
   <si>
-    <t>ready</t>
-  </si>
-  <si>
     <t>semi finished</t>
   </si>
   <si>
@@ -206,6 +203,9 @@
   </si>
   <si>
     <t>pp5_installment_amount_yearly2</t>
+  </si>
+  <si>
+    <t>ready to move</t>
   </si>
 </sst>
 </file>
@@ -1854,97 +1854,97 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="D1" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="E1" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="G1" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="H1" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="I1" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="J1" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="K1" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="L1" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="M1" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="N1" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="O1" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="O1" s="4" t="s">
+      <c r="P1" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="P1" s="4" t="s">
+      <c r="Q1" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="Q1" s="4" t="s">
+      <c r="R1" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="R1" s="4" t="s">
+      <c r="S1" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="S1" s="4" t="s">
+      <c r="T1" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="T1" s="4" t="s">
+      <c r="U1" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="U1" s="4" t="s">
+      <c r="V1" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="V1" s="4" t="s">
+      <c r="W1" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="W1" s="4" t="s">
+      <c r="X1" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="X1" s="4" t="s">
+      <c r="Y1" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="Y1" s="4" t="s">
+      <c r="Z1" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="Z1" s="4" t="s">
+      <c r="AA1" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="AA1" s="4" t="s">
+      <c r="AB1" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="AB1" s="4" t="s">
+      <c r="AC1" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="AC1" s="4" t="s">
+      <c r="AD1" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="AD1" s="4" t="s">
+      <c r="AE1" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="AE1" s="4" t="s">
+      <c r="AF1" s="4" t="s">
         <v>60</v>
-      </c>
-      <c r="AF1" s="4" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:32" ht="15.6" x14ac:dyDescent="0.3">
@@ -2072,7 +2072,7 @@
         <v>24</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>25</v>
+        <v>61</v>
       </c>
       <c r="K3" s="3">
         <v>2</v>
@@ -2090,20 +2090,20 @@
         <v>20</v>
       </c>
       <c r="P3" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q3" s="3" t="s">
         <v>26</v>
-      </c>
-      <c r="Q3" s="3" t="s">
-        <v>27</v>
       </c>
       <c r="R3" s="3">
         <v>1</v>
       </c>
       <c r="S3" s="5"/>
       <c r="T3" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="U3" s="3" t="s">
         <v>28</v>
-      </c>
-      <c r="U3" s="3" t="s">
-        <v>29</v>
       </c>
       <c r="V3" s="3">
         <v>500000</v>
@@ -2112,7 +2112,7 @@
         <v>4200000</v>
       </c>
       <c r="X3" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Y3" s="3">
         <v>300000</v>

</xml_diff>